<commit_message>
Data filter & Spearman
</commit_message>
<xml_diff>
--- a/casebase/statistics/record.xlsx
+++ b/casebase/statistics/record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\0_code\block-gml-casebase\casebase\statistics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{791DFB1D-2EA4-46AE-A494-1827285081A3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1E737B7-05CC-4BEF-AC0F-4BE8FA43559A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="25824" windowHeight="15504" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="178">
   <si>
     <t>city</t>
   </si>
@@ -553,6 +553,10 @@
   </si>
   <si>
     <t>1.2（1.3）</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>截断数据后lod1</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1063,7 +1067,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P35"/>
+  <dimension ref="A1:Q35"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" style="1" customWidth="1"/>
@@ -1081,7 +1085,7 @@
     <col min="18" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="41.4" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" ht="41.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1130,8 +1134,11 @@
       <c r="P1" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q1" s="1" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>14</v>
       </c>
@@ -1184,8 +1191,11 @@
         <f>SUM(L2:L46)</f>
         <v>46276</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q2" s="1">
+        <v>181858</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>19</v>
       </c>
@@ -1223,7 +1233,7 @@
         <v>5571</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>22</v>
       </c>
@@ -1261,7 +1271,7 @@
         <v>2957</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>25</v>
       </c>
@@ -1293,7 +1303,7 @@
         <v>1498</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>29</v>
       </c>
@@ -1331,7 +1341,7 @@
         <v>1253</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>32</v>
       </c>
@@ -1369,7 +1379,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>34</v>
       </c>
@@ -1401,7 +1411,7 @@
         <v>1899</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>36</v>
       </c>
@@ -1433,7 +1443,7 @@
         <v>879</v>
       </c>
     </row>
-    <row r="10" spans="1:16" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>38</v>
       </c>
@@ -1462,7 +1472,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>41</v>
       </c>
@@ -1494,7 +1504,7 @@
         <v>4700</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>44</v>
       </c>
@@ -1532,7 +1542,7 @@
         <v>2154</v>
       </c>
     </row>
-    <row r="13" spans="1:16" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
         <v>46</v>
       </c>
@@ -1567,7 +1577,7 @@
         <v>2598</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>49</v>
       </c>
@@ -1605,7 +1615,7 @@
         <v>2650</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>51</v>
       </c>
@@ -1643,7 +1653,7 @@
         <v>8762</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>53</v>
       </c>
@@ -2415,15 +2425,15 @@
       </c>
       <c r="P2" s="12">
         <f>SUM(G2:G31)</f>
-        <v>13621448</v>
+        <v>13621447</v>
       </c>
       <c r="Q2" s="12">
         <f>SUM(H2:H31)</f>
-        <v>146566833</v>
+        <v>146597931</v>
       </c>
       <c r="R2" s="12">
         <f>SUM(J2:J31)</f>
-        <v>12187283</v>
+        <v>12187282</v>
       </c>
       <c r="S2" s="12">
         <f>SUM(K2:K30)</f>
@@ -2435,7 +2445,7 @@
       <c r="X2" s="1"/>
       <c r="Y2" s="1"/>
     </row>
-    <row r="3" spans="1:25" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>22</v>
       </c>
@@ -2531,16 +2541,16 @@
         <v>123</v>
       </c>
       <c r="G5" s="3">
-        <v>928003</v>
+        <v>928002</v>
       </c>
       <c r="H5" s="3">
-        <v>9805809</v>
+        <v>9836907</v>
       </c>
       <c r="I5" s="3">
         <v>25833</v>
       </c>
       <c r="J5" s="3">
-        <v>844938</v>
+        <v>844937</v>
       </c>
       <c r="K5" s="3">
         <v>6.6</v>

</xml_diff>